<commit_message>
WROTE ALL TILL EMPIRICAL APPLICATION
</commit_message>
<xml_diff>
--- a/data/controles_results/dif_medias/controls_staggered_vars/difmedias_controles_staggered_variables_2015_T1_0.xlsx
+++ b/data/controles_results/dif_medias/controls_staggered_vars/difmedias_controles_staggered_variables_2015_T1_0.xlsx
@@ -45,7 +45,7 @@
     <t>N</t>
   </si>
   <si>
-    <t>94</t>
+    <t>90</t>
   </si>
   <si>
     <t xml:space="preserve"> (1) </t>
@@ -63,16 +63,16 @@
     <t>(0.000)</t>
   </si>
   <si>
-    <t>0.138</t>
-  </si>
-  <si>
-    <t>(0.036)</t>
-  </si>
-  <si>
-    <t>0.181</t>
-  </si>
-  <si>
-    <t>(0.050)</t>
+    <t>0.144</t>
+  </si>
+  <si>
+    <t>(0.037)</t>
+  </si>
+  <si>
+    <t>0.189</t>
+  </si>
+  <si>
+    <t>(0.052)</t>
   </si>
   <si>
     <t>20</t>
@@ -99,7 +99,7 @@
     <t>.n</t>
   </si>
   <si>
-    <t>114</t>
+    <t>110</t>
   </si>
   <si>
     <t>(2)-(1)</t>
@@ -111,10 +111,10 @@
     <t>Mean difference</t>
   </si>
   <si>
-    <t>0.262***</t>
-  </si>
-  <si>
-    <t>0.469***</t>
+    <t>0.256***</t>
+  </si>
+  <si>
+    <t>0.461***</t>
   </si>
 </sst>
 </file>

</xml_diff>